<commit_message>
fix(medios): sincroniza catalogo canonico de 106 fuentes
</commit_message>
<xml_diff>
--- a/centro-local/data/medios/Medios_Matriz_Geopolitica_Navegacion_actualizado.xlsx
+++ b/centro-local/data/medios/Medios_Matriz_Geopolitica_Navegacion_actualizado.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R26d67655b1e4471d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriz profesional" sheetId="2" r:id="R64cedb75a79b4c4c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metodología" sheetId="3" r:id="R8fc906fb48264811"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Original" sheetId="4" r:id="Rf0fb99a224314174"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura África" sheetId="5" r:id="R0f64968c9d2c4b79"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Por Región" sheetId="6" r:id="R558c358d66604682"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Por Función" sheetId="7" r:id="R9e31d173e23c4d52"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Por Perspectiva" sheetId="8" r:id="Rc67c8fdff8ad46a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consulta rápida" sheetId="9" r:id="Rbf458d6e36204b34"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Re92841ca88bb4fa5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriz profesional" sheetId="2" r:id="R1a41b432a666489b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metodología" sheetId="3" r:id="Re27ec3dacb934745"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Original" sheetId="4" r:id="R70a893e5b1d74a13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura África" sheetId="5" r:id="R8fffe0ce2db04e48"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Por Región" sheetId="6" r:id="R2a891143477f4338"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Por Función" sheetId="7" r:id="Rb69b787360be4d26"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Por Perspectiva" sheetId="8" r:id="R5aaa21cd88634ab8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consulta rápida" sheetId="9" r:id="R903cef7aea4240f0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1750,9 +1750,7 @@
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="48672768"/>
         <c:crosses val="autoZero"/>
-        <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
-        <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
         <c:axId val="48672768"/>
@@ -1875,9 +1873,7 @@
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="48672768"/>
         <c:crosses val="autoZero"/>
-        <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
-        <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
         <c:axId val="48672768"/>
@@ -2000,9 +1996,7 @@
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="48672768"/>
         <c:crosses val="autoZero"/>
-        <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
-        <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
         <c:axId val="48672768"/>
@@ -2068,7 +2062,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb7c517d4863749ed"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7694a7d5a2de4c83"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2098,7 +2092,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R09e201f83a8c4968"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Racbe43e70939475f"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2133,7 +2127,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3caf40cd0702496d"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7fd4d805c5cd4ff7"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2493,7 +2487,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="85" t="str">
-        <x:v>Resumen automático de la matriz. Los indicadores reflejan la evaluación preliminar del 16/07/2026.</x:v>
+        <x:v>Resumen automático de la matriz. Se incorporaron 13 fuentes propuestas el 26/08/2026; sus valoraciones quedan pendientes de revisión editorial.</x:v>
       </x:c>
       <x:c r="B2" s="85"/>
       <x:c r="C2" s="85"/>
@@ -2530,7 +2524,7 @@
         <x:v>Total de fuentes</x:v>
       </x:c>
       <x:c r="B5" s="101" t="n">
-        <x:v>93</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="D5" s="117" t="str">
         <x:v>Alta</x:v>
@@ -2644,6 +2638,18 @@
       <x:c r="B10" s="101" t="n">
         <x:f>COUNTIF('Matriz profesional'!X5:X96,"Secundario")</x:f>
         <x:v>2</x:v>
+      </x:c>
+      <x:c r="D10" t="str">
+        <x:v>Por revisar</x:v>
+      </x:c>
+      <x:c r="E10" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="G10" t="str">
+        <x:v>Propuesto</x:v>
+      </x:c>
+      <x:c r="H10" t="n">
+        <x:v>13</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -2842,7 +2848,7 @@
     <x:mergeCell ref="B34:J34"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8366f6259e294831"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d7481a8c5dc4762"/>
 </x:worksheet>
 </file>
 
@@ -3023,6 +3029,9 @@
       <x:c r="AA4" s="33" t="str">
         <x:v>Fecha de revisión</x:v>
       </x:c>
+      <x:c r="AB4" t="str">
+        <x:v>Media ID estable</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="60" t="n">
@@ -10819,6 +10828,994 @@
       </x:c>
       <x:c r="AA97" t="n">
         <x:v>46229</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98">
+      <x:c r="A98" t="n">
+        <x:v>94</x:v>
+      </x:c>
+      <x:c r="B98" t="str">
+        <x:v>Carnegie Endowment for International Peace</x:v>
+      </x:c>
+      <x:c r="C98" t="str">
+        <x:v>https://carnegieendowment.org/</x:v>
+      </x:c>
+      <x:c r="D98" t="str"/>
+      <x:c r="E98" t="str">
+        <x:v>Global/Occidente</x:v>
+      </x:c>
+      <x:c r="F98" t="str">
+        <x:v>Multilingüe</x:v>
+      </x:c>
+      <x:c r="G98" t="str">
+        <x:v>Think tank</x:v>
+      </x:c>
+      <x:c r="H98" t="str">
+        <x:v>Análisis de política internacional</x:v>
+      </x:c>
+      <x:c r="I98" t="str"/>
+      <x:c r="J98" t="str"/>
+      <x:c r="K98" t="str"/>
+      <x:c r="L98" t="str">
+        <x:v>Estadounidense / internacionalista</x:v>
+      </x:c>
+      <x:c r="M98" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N98" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O98" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P98" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q98" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R98" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S98" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T98" t="str">
+        <x:v>Por revisar</x:v>
+      </x:c>
+      <x:c r="U98" t="str">
+        <x:v>Fuente incorporada para seguimiento editorial.</x:v>
+      </x:c>
+      <x:c r="V98" t="str">
+        <x:v>Corroborar afirmaciones sensibles con otra familia de fuentes.</x:v>
+      </x:c>
+      <x:c r="W98" t="str"/>
+      <x:c r="X98" t="str">
+        <x:v>propuesto</x:v>
+      </x:c>
+      <x:c r="Y98" t="str">
+        <x:v>Alta asistida durante la preparación de macroeventos sobre Turquía.</x:v>
+      </x:c>
+      <x:c r="Z98" t="str">
+        <x:v>https://carnegieendowment.org/</x:v>
+      </x:c>
+      <x:c r="AA98" t="n">
+        <x:v>46260</x:v>
+      </x:c>
+      <x:c r="AB98" t="str">
+        <x:v>carnegie-endowment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99">
+      <x:c r="A99" t="n">
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="B99" t="str">
+        <x:v>U.S. Department of Defense</x:v>
+      </x:c>
+      <x:c r="C99" t="str">
+        <x:v>https://www.defense.gov/</x:v>
+      </x:c>
+      <x:c r="D99" t="str"/>
+      <x:c r="E99" t="str">
+        <x:v>Global</x:v>
+      </x:c>
+      <x:c r="F99" t="str">
+        <x:v>Multilingüe</x:v>
+      </x:c>
+      <x:c r="G99" t="str">
+        <x:v>Agencia gubernamental</x:v>
+      </x:c>
+      <x:c r="H99" t="str">
+        <x:v>Documentación y supervisión de defensa</x:v>
+      </x:c>
+      <x:c r="I99" t="str"/>
+      <x:c r="J99" t="str"/>
+      <x:c r="K99" t="str"/>
+      <x:c r="L99" t="str">
+        <x:v>Estadounidense / militar</x:v>
+      </x:c>
+      <x:c r="M99" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N99" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O99" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P99" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q99" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R99" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S99" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T99" t="str">
+        <x:v>Por revisar</x:v>
+      </x:c>
+      <x:c r="U99" t="str">
+        <x:v>Fuente incorporada para seguimiento editorial.</x:v>
+      </x:c>
+      <x:c r="V99" t="str">
+        <x:v>Corroborar afirmaciones sensibles con otra familia de fuentes.</x:v>
+      </x:c>
+      <x:c r="W99" t="str"/>
+      <x:c r="X99" t="str">
+        <x:v>propuesto</x:v>
+      </x:c>
+      <x:c r="Y99" t="str">
+        <x:v>Alta asistida durante la preparación de macroeventos sobre Turquía.</x:v>
+      </x:c>
+      <x:c r="Z99" t="str">
+        <x:v>https://www.defense.gov/</x:v>
+      </x:c>
+      <x:c r="AA99" t="n">
+        <x:v>46260</x:v>
+      </x:c>
+      <x:c r="AB99" t="str">
+        <x:v>us-department-defense</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100">
+      <x:c r="A100" t="n">
+        <x:v>96</x:v>
+      </x:c>
+      <x:c r="B100" t="str">
+        <x:v>Brookings Institution</x:v>
+      </x:c>
+      <x:c r="C100" t="str">
+        <x:v>https://www.brookings.edu/</x:v>
+      </x:c>
+      <x:c r="D100" t="str"/>
+      <x:c r="E100" t="str">
+        <x:v>Global/Occidente</x:v>
+      </x:c>
+      <x:c r="F100" t="str">
+        <x:v>Multilingüe</x:v>
+      </x:c>
+      <x:c r="G100" t="str">
+        <x:v>Think tank</x:v>
+      </x:c>
+      <x:c r="H100" t="str">
+        <x:v>Investigación y análisis de políticas</x:v>
+      </x:c>
+      <x:c r="I100" t="str"/>
+      <x:c r="J100" t="str"/>
+      <x:c r="K100" t="str"/>
+      <x:c r="L100" t="str">
+        <x:v>Estadounidense / política pública</x:v>
+      </x:c>
+      <x:c r="M100" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N100" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O100" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P100" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q100" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R100" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S100" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T100" t="str">
+        <x:v>Por revisar</x:v>
+      </x:c>
+      <x:c r="U100" t="str">
+        <x:v>Fuente incorporada para seguimiento editorial.</x:v>
+      </x:c>
+      <x:c r="V100" t="str">
+        <x:v>Corroborar afirmaciones sensibles con otra familia de fuentes.</x:v>
+      </x:c>
+      <x:c r="W100" t="str"/>
+      <x:c r="X100" t="str">
+        <x:v>propuesto</x:v>
+      </x:c>
+      <x:c r="Y100" t="str">
+        <x:v>Alta asistida durante la preparación de macroeventos sobre Turquía.</x:v>
+      </x:c>
+      <x:c r="Z100" t="str">
+        <x:v>https://www.brookings.edu/</x:v>
+      </x:c>
+      <x:c r="AA100" t="n">
+        <x:v>46260</x:v>
+      </x:c>
+      <x:c r="AB100" t="str">
+        <x:v>brookings-institution</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101">
+      <x:c r="A101" t="n">
+        <x:v>97</x:v>
+      </x:c>
+      <x:c r="B101" t="str">
+        <x:v>Anadolu Agency</x:v>
+      </x:c>
+      <x:c r="C101" t="str">
+        <x:v>https://www.aa.com.tr/</x:v>
+      </x:c>
+      <x:c r="D101" t="str"/>
+      <x:c r="E101" t="str">
+        <x:v>Turquía/Global</x:v>
+      </x:c>
+      <x:c r="F101" t="str">
+        <x:v>Multilingüe</x:v>
+      </x:c>
+      <x:c r="G101" t="str">
+        <x:v>Agencia estatal de noticias</x:v>
+      </x:c>
+      <x:c r="H101" t="str">
+        <x:v>Noticias, entrevistas y comunicados</x:v>
+      </x:c>
+      <x:c r="I101" t="str"/>
+      <x:c r="J101" t="str"/>
+      <x:c r="K101" t="str"/>
+      <x:c r="L101" t="str">
+        <x:v>Turca / estatal</x:v>
+      </x:c>
+      <x:c r="M101" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N101" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O101" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P101" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q101" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R101" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S101" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T101" t="str">
+        <x:v>Por revisar</x:v>
+      </x:c>
+      <x:c r="U101" t="str">
+        <x:v>Fuente incorporada para seguimiento editorial.</x:v>
+      </x:c>
+      <x:c r="V101" t="str">
+        <x:v>Corroborar afirmaciones sensibles con otra familia de fuentes.</x:v>
+      </x:c>
+      <x:c r="W101" t="str"/>
+      <x:c r="X101" t="str">
+        <x:v>propuesto</x:v>
+      </x:c>
+      <x:c r="Y101" t="str">
+        <x:v>Alta asistida durante la preparación de macroeventos sobre Turquía.</x:v>
+      </x:c>
+      <x:c r="Z101" t="str">
+        <x:v>https://www.aa.com.tr/</x:v>
+      </x:c>
+      <x:c r="AA101" t="n">
+        <x:v>46260</x:v>
+      </x:c>
+      <x:c r="AB101" t="str">
+        <x:v>anadolu-agency</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="102">
+      <x:c r="A102" t="n">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="B102" t="str">
+        <x:v>Le Monde</x:v>
+      </x:c>
+      <x:c r="C102" t="str">
+        <x:v>https://www.lemonde.fr/</x:v>
+      </x:c>
+      <x:c r="D102" t="str"/>
+      <x:c r="E102" t="str">
+        <x:v>Europa/Global</x:v>
+      </x:c>
+      <x:c r="F102" t="str">
+        <x:v>Multilingüe</x:v>
+      </x:c>
+      <x:c r="G102" t="str">
+        <x:v>Medio generalista</x:v>
+      </x:c>
+      <x:c r="H102" t="str">
+        <x:v>Información y análisis internacional</x:v>
+      </x:c>
+      <x:c r="I102" t="str"/>
+      <x:c r="J102" t="str"/>
+      <x:c r="K102" t="str"/>
+      <x:c r="L102" t="str">
+        <x:v>Francesa / europea</x:v>
+      </x:c>
+      <x:c r="M102" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N102" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O102" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P102" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q102" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R102" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S102" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T102" t="str">
+        <x:v>Por revisar</x:v>
+      </x:c>
+      <x:c r="U102" t="str">
+        <x:v>Fuente incorporada para seguimiento editorial.</x:v>
+      </x:c>
+      <x:c r="V102" t="str">
+        <x:v>Corroborar afirmaciones sensibles con otra familia de fuentes.</x:v>
+      </x:c>
+      <x:c r="W102" t="str"/>
+      <x:c r="X102" t="str">
+        <x:v>propuesto</x:v>
+      </x:c>
+      <x:c r="Y102" t="str">
+        <x:v>Alta asistida durante la preparación de macroeventos sobre Turquía.</x:v>
+      </x:c>
+      <x:c r="Z102" t="str">
+        <x:v>https://www.lemonde.fr/</x:v>
+      </x:c>
+      <x:c r="AA102" t="n">
+        <x:v>46260</x:v>
+      </x:c>
+      <x:c r="AB102" t="str">
+        <x:v>le-monde</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="103">
+      <x:c r="A103" t="n">
+        <x:v>99</x:v>
+      </x:c>
+      <x:c r="B103" t="str">
+        <x:v>Secretariat of Defence Industries (SSB)</x:v>
+      </x:c>
+      <x:c r="C103" t="str">
+        <x:v>https://www.ssb.gov.tr/</x:v>
+      </x:c>
+      <x:c r="D103" t="str"/>
+      <x:c r="E103" t="str">
+        <x:v>Turquía</x:v>
+      </x:c>
+      <x:c r="F103" t="str">
+        <x:v>Multilingüe</x:v>
+      </x:c>
+      <x:c r="G103" t="str">
+        <x:v>Agencia gubernamental</x:v>
+      </x:c>
+      <x:c r="H103" t="str">
+        <x:v>Datos y comunicados oficiales del sector</x:v>
+      </x:c>
+      <x:c r="I103" t="str"/>
+      <x:c r="J103" t="str"/>
+      <x:c r="K103" t="str"/>
+      <x:c r="L103" t="str">
+        <x:v>Turca / industria de defensa</x:v>
+      </x:c>
+      <x:c r="M103" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N103" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O103" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P103" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q103" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R103" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S103" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T103" t="str">
+        <x:v>Por revisar</x:v>
+      </x:c>
+      <x:c r="U103" t="str">
+        <x:v>Fuente incorporada para seguimiento editorial.</x:v>
+      </x:c>
+      <x:c r="V103" t="str">
+        <x:v>Corroborar afirmaciones sensibles con otra familia de fuentes.</x:v>
+      </x:c>
+      <x:c r="W103" t="str"/>
+      <x:c r="X103" t="str">
+        <x:v>propuesto</x:v>
+      </x:c>
+      <x:c r="Y103" t="str">
+        <x:v>Alta asistida durante la preparación de macroeventos sobre Turquía.</x:v>
+      </x:c>
+      <x:c r="Z103" t="str">
+        <x:v>https://www.ssb.gov.tr/</x:v>
+      </x:c>
+      <x:c r="AA103" t="n">
+        <x:v>46260</x:v>
+      </x:c>
+      <x:c r="AB103" t="str">
+        <x:v>turkiye-ssb</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="104">
+      <x:c r="A104" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="B104" t="str">
+        <x:v>TotalEnergies</x:v>
+      </x:c>
+      <x:c r="C104" t="str">
+        <x:v>https://totalenergies.com/</x:v>
+      </x:c>
+      <x:c r="D104" t="str"/>
+      <x:c r="E104" t="str">
+        <x:v>Global/Europa</x:v>
+      </x:c>
+      <x:c r="F104" t="str">
+        <x:v>Multilingüe</x:v>
+      </x:c>
+      <x:c r="G104" t="str">
+        <x:v>Fuente corporativa</x:v>
+      </x:c>
+      <x:c r="H104" t="str">
+        <x:v>Información primaria sobre proyectos propios</x:v>
+      </x:c>
+      <x:c r="I104" t="str"/>
+      <x:c r="J104" t="str"/>
+      <x:c r="K104" t="str"/>
+      <x:c r="L104" t="str">
+        <x:v>Corporativa / energética</x:v>
+      </x:c>
+      <x:c r="M104" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N104" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O104" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P104" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q104" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R104" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S104" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T104" t="str">
+        <x:v>Por revisar</x:v>
+      </x:c>
+      <x:c r="U104" t="str">
+        <x:v>Fuente incorporada para seguimiento editorial.</x:v>
+      </x:c>
+      <x:c r="V104" t="str">
+        <x:v>Corroborar afirmaciones sensibles con otra familia de fuentes.</x:v>
+      </x:c>
+      <x:c r="W104" t="str"/>
+      <x:c r="X104" t="str">
+        <x:v>propuesto</x:v>
+      </x:c>
+      <x:c r="Y104" t="str">
+        <x:v>Alta asistida durante la preparación de macroeventos sobre Turquía.</x:v>
+      </x:c>
+      <x:c r="Z104" t="str">
+        <x:v>https://totalenergies.com/</x:v>
+      </x:c>
+      <x:c r="AA104" t="n">
+        <x:v>46260</x:v>
+      </x:c>
+      <x:c r="AB104" t="str">
+        <x:v>totalenergies</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="105">
+      <x:c r="A105" t="n">
+        <x:v>101</x:v>
+      </x:c>
+      <x:c r="B105" t="str">
+        <x:v>Eni</x:v>
+      </x:c>
+      <x:c r="C105" t="str">
+        <x:v>https://www.eni.com/</x:v>
+      </x:c>
+      <x:c r="D105" t="str"/>
+      <x:c r="E105" t="str">
+        <x:v>Global/Europa</x:v>
+      </x:c>
+      <x:c r="F105" t="str">
+        <x:v>Multilingüe</x:v>
+      </x:c>
+      <x:c r="G105" t="str">
+        <x:v>Fuente corporativa</x:v>
+      </x:c>
+      <x:c r="H105" t="str">
+        <x:v>Información primaria sobre proyectos propios</x:v>
+      </x:c>
+      <x:c r="I105" t="str"/>
+      <x:c r="J105" t="str"/>
+      <x:c r="K105" t="str"/>
+      <x:c r="L105" t="str">
+        <x:v>Corporativa / energética</x:v>
+      </x:c>
+      <x:c r="M105" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N105" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O105" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P105" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q105" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R105" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S105" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T105" t="str">
+        <x:v>Por revisar</x:v>
+      </x:c>
+      <x:c r="U105" t="str">
+        <x:v>Fuente incorporada para seguimiento editorial.</x:v>
+      </x:c>
+      <x:c r="V105" t="str">
+        <x:v>Corroborar afirmaciones sensibles con otra familia de fuentes.</x:v>
+      </x:c>
+      <x:c r="W105" t="str"/>
+      <x:c r="X105" t="str">
+        <x:v>propuesto</x:v>
+      </x:c>
+      <x:c r="Y105" t="str">
+        <x:v>Alta asistida durante la preparación de macroeventos sobre Turquía.</x:v>
+      </x:c>
+      <x:c r="Z105" t="str">
+        <x:v>https://www.eni.com/</x:v>
+      </x:c>
+      <x:c r="AA105" t="n">
+        <x:v>46260</x:v>
+      </x:c>
+      <x:c r="AB105" t="str">
+        <x:v>eni</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="106">
+      <x:c r="A106" t="n">
+        <x:v>102</x:v>
+      </x:c>
+      <x:c r="B106" t="str">
+        <x:v>Italian Ministry of Foreign Affairs and International Cooperation</x:v>
+      </x:c>
+      <x:c r="C106" t="str">
+        <x:v>https://www.esteri.it/</x:v>
+      </x:c>
+      <x:c r="D106" t="str"/>
+      <x:c r="E106" t="str">
+        <x:v>Europa</x:v>
+      </x:c>
+      <x:c r="F106" t="str">
+        <x:v>Multilingüe</x:v>
+      </x:c>
+      <x:c r="G106" t="str">
+        <x:v>Ministerio gubernamental</x:v>
+      </x:c>
+      <x:c r="H106" t="str">
+        <x:v>Información oficial y diplomacia económica</x:v>
+      </x:c>
+      <x:c r="I106" t="str"/>
+      <x:c r="J106" t="str"/>
+      <x:c r="K106" t="str"/>
+      <x:c r="L106" t="str">
+        <x:v>Italiana / diplomacia económica</x:v>
+      </x:c>
+      <x:c r="M106" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N106" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O106" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P106" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q106" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R106" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S106" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T106" t="str">
+        <x:v>Por revisar</x:v>
+      </x:c>
+      <x:c r="U106" t="str">
+        <x:v>Fuente incorporada para seguimiento editorial.</x:v>
+      </x:c>
+      <x:c r="V106" t="str">
+        <x:v>Corroborar afirmaciones sensibles con otra familia de fuentes.</x:v>
+      </x:c>
+      <x:c r="W106" t="str"/>
+      <x:c r="X106" t="str">
+        <x:v>propuesto</x:v>
+      </x:c>
+      <x:c r="Y106" t="str">
+        <x:v>Alta asistida durante la preparación de macroeventos sobre Turquía.</x:v>
+      </x:c>
+      <x:c r="Z106" t="str">
+        <x:v>https://www.esteri.it/</x:v>
+      </x:c>
+      <x:c r="AA106" t="n">
+        <x:v>46260</x:v>
+      </x:c>
+      <x:c r="AB106" t="str">
+        <x:v>italian-foreign-ministry</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="107">
+      <x:c r="A107" t="n">
+        <x:v>103</x:v>
+      </x:c>
+      <x:c r="B107" t="str">
+        <x:v>Middle East Council on Global Affairs</x:v>
+      </x:c>
+      <x:c r="C107" t="str">
+        <x:v>https://mecouncil.org/</x:v>
+      </x:c>
+      <x:c r="D107" t="str"/>
+      <x:c r="E107" t="str">
+        <x:v>Medio Oriente</x:v>
+      </x:c>
+      <x:c r="F107" t="str">
+        <x:v>Multilingüe</x:v>
+      </x:c>
+      <x:c r="G107" t="str">
+        <x:v>Think tank</x:v>
+      </x:c>
+      <x:c r="H107" t="str">
+        <x:v>Investigación de política regional</x:v>
+      </x:c>
+      <x:c r="I107" t="str"/>
+      <x:c r="J107" t="str"/>
+      <x:c r="K107" t="str"/>
+      <x:c r="L107" t="str">
+        <x:v>Regional / Golfo</x:v>
+      </x:c>
+      <x:c r="M107" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N107" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O107" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P107" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q107" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R107" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S107" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T107" t="str">
+        <x:v>Por revisar</x:v>
+      </x:c>
+      <x:c r="U107" t="str">
+        <x:v>Fuente incorporada para seguimiento editorial.</x:v>
+      </x:c>
+      <x:c r="V107" t="str">
+        <x:v>Corroborar afirmaciones sensibles con otra familia de fuentes.</x:v>
+      </x:c>
+      <x:c r="W107" t="str"/>
+      <x:c r="X107" t="str">
+        <x:v>propuesto</x:v>
+      </x:c>
+      <x:c r="Y107" t="str">
+        <x:v>Alta asistida durante la preparación de macroeventos sobre Turquía.</x:v>
+      </x:c>
+      <x:c r="Z107" t="str">
+        <x:v>https://mecouncil.org/</x:v>
+      </x:c>
+      <x:c r="AA107" t="n">
+        <x:v>46260</x:v>
+      </x:c>
+      <x:c r="AB107" t="str">
+        <x:v>middle-east-council-global-affairs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108">
+      <x:c r="A108" t="n">
+        <x:v>104</x:v>
+      </x:c>
+      <x:c r="B108" t="str">
+        <x:v>Iraqi News Agency (INA)</x:v>
+      </x:c>
+      <x:c r="C108" t="str">
+        <x:v>https://ina.iq/</x:v>
+      </x:c>
+      <x:c r="D108" t="str"/>
+      <x:c r="E108" t="str">
+        <x:v>Medio Oriente</x:v>
+      </x:c>
+      <x:c r="F108" t="str">
+        <x:v>Multilingüe</x:v>
+      </x:c>
+      <x:c r="G108" t="str">
+        <x:v>Agencia estatal de noticias</x:v>
+      </x:c>
+      <x:c r="H108" t="str">
+        <x:v>Información oficial y noticias nacionales</x:v>
+      </x:c>
+      <x:c r="I108" t="str"/>
+      <x:c r="J108" t="str"/>
+      <x:c r="K108" t="str"/>
+      <x:c r="L108" t="str">
+        <x:v>Iraquí / estatal</x:v>
+      </x:c>
+      <x:c r="M108" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N108" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O108" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P108" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q108" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R108" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S108" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T108" t="str">
+        <x:v>Por revisar</x:v>
+      </x:c>
+      <x:c r="U108" t="str">
+        <x:v>Fuente incorporada para seguimiento editorial.</x:v>
+      </x:c>
+      <x:c r="V108" t="str">
+        <x:v>Corroborar afirmaciones sensibles con otra familia de fuentes.</x:v>
+      </x:c>
+      <x:c r="W108" t="str"/>
+      <x:c r="X108" t="str">
+        <x:v>propuesto</x:v>
+      </x:c>
+      <x:c r="Y108" t="str">
+        <x:v>Alta asistida durante la preparación de macroeventos sobre Turquía.</x:v>
+      </x:c>
+      <x:c r="Z108" t="str">
+        <x:v>https://ina.iq/</x:v>
+      </x:c>
+      <x:c r="AA108" t="n">
+        <x:v>46260</x:v>
+      </x:c>
+      <x:c r="AB108" t="str">
+        <x:v>iraqi-news-agency</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109">
+      <x:c r="A109" t="n">
+        <x:v>105</x:v>
+      </x:c>
+      <x:c r="B109" t="str">
+        <x:v>Republic of Türkiye Ministry of Energy and Natural Resources</x:v>
+      </x:c>
+      <x:c r="C109" t="str">
+        <x:v>https://enerji.gov.tr/</x:v>
+      </x:c>
+      <x:c r="D109" t="str"/>
+      <x:c r="E109" t="str">
+        <x:v>Turquía</x:v>
+      </x:c>
+      <x:c r="F109" t="str">
+        <x:v>Multilingüe</x:v>
+      </x:c>
+      <x:c r="G109" t="str">
+        <x:v>Ministerio gubernamental</x:v>
+      </x:c>
+      <x:c r="H109" t="str">
+        <x:v>Datos y comunicados oficiales de energía</x:v>
+      </x:c>
+      <x:c r="I109" t="str"/>
+      <x:c r="J109" t="str"/>
+      <x:c r="K109" t="str"/>
+      <x:c r="L109" t="str">
+        <x:v>Turca / energética</x:v>
+      </x:c>
+      <x:c r="M109" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N109" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O109" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P109" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q109" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R109" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S109" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T109" t="str">
+        <x:v>Por revisar</x:v>
+      </x:c>
+      <x:c r="U109" t="str">
+        <x:v>Fuente incorporada para seguimiento editorial.</x:v>
+      </x:c>
+      <x:c r="V109" t="str">
+        <x:v>Corroborar afirmaciones sensibles con otra familia de fuentes.</x:v>
+      </x:c>
+      <x:c r="W109" t="str"/>
+      <x:c r="X109" t="str">
+        <x:v>propuesto</x:v>
+      </x:c>
+      <x:c r="Y109" t="str">
+        <x:v>Alta asistida durante la preparación de macroeventos sobre Turquía.</x:v>
+      </x:c>
+      <x:c r="Z109" t="str">
+        <x:v>https://enerji.gov.tr/</x:v>
+      </x:c>
+      <x:c r="AA109" t="n">
+        <x:v>46260</x:v>
+      </x:c>
+      <x:c r="AB109" t="str">
+        <x:v>turkiye-energy-ministry</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="110">
+      <x:c r="A110" t="n">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="B110" t="str">
+        <x:v>The Washington Institute for Near East Policy</x:v>
+      </x:c>
+      <x:c r="C110" t="str">
+        <x:v>https://www.washingtoninstitute.org/</x:v>
+      </x:c>
+      <x:c r="D110" t="str"/>
+      <x:c r="E110" t="str">
+        <x:v>Estados Unidos/Medio Oriente</x:v>
+      </x:c>
+      <x:c r="F110" t="str">
+        <x:v>Multilingüe</x:v>
+      </x:c>
+      <x:c r="G110" t="str">
+        <x:v>Think tank</x:v>
+      </x:c>
+      <x:c r="H110" t="str">
+        <x:v>Análisis de seguridad y política regional</x:v>
+      </x:c>
+      <x:c r="I110" t="str"/>
+      <x:c r="J110" t="str"/>
+      <x:c r="K110" t="str"/>
+      <x:c r="L110" t="str">
+        <x:v>Estadounidense / seguridad regional</x:v>
+      </x:c>
+      <x:c r="M110" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N110" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O110" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P110" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q110" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R110" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S110" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T110" t="str">
+        <x:v>Por revisar</x:v>
+      </x:c>
+      <x:c r="U110" t="str">
+        <x:v>Fuente incorporada para seguimiento editorial.</x:v>
+      </x:c>
+      <x:c r="V110" t="str">
+        <x:v>Corroborar afirmaciones sensibles con otra familia de fuentes.</x:v>
+      </x:c>
+      <x:c r="W110" t="str"/>
+      <x:c r="X110" t="str">
+        <x:v>propuesto</x:v>
+      </x:c>
+      <x:c r="Y110" t="str">
+        <x:v>Alta asistida durante la preparación de macroeventos sobre Turquía.</x:v>
+      </x:c>
+      <x:c r="Z110" t="str">
+        <x:v>https://www.washingtoninstitute.org/</x:v>
+      </x:c>
+      <x:c r="AA110" t="n">
+        <x:v>46260</x:v>
+      </x:c>
+      <x:c r="AB110" t="str">
+        <x:v>washington-institute</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -10932,7 +11929,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5a001b784d544a4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re6ff8bbf627b45c5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14245,9 +15242,9 @@
     <x:mergeCell ref="A38:H40"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18be216a45d64b75"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R34b8d042bb3042a4"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd67d59710ec94782"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f92bd6619084238"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22050,7 +23047,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R854b35b2779e43ce"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R65790e2480984c7e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -29853,7 +30850,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd459cf22c2d04d20"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reea4b2f248614ea3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -37656,7 +38653,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R78d540c9d7974ee9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e96e870eae2490c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -41290,7 +42287,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0d7ffa9101704361"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c977073c5d846ba"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>